<commit_message>
Fix param_tuning pipeline analysis
</commit_message>
<xml_diff>
--- a/param_tuning/20250927-datasets.xlsx
+++ b/param_tuning/20250927-datasets.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="92">
   <si>
     <t xml:space="preserve">BEST Pipelines</t>
   </si>
@@ -282,9 +282,6 @@
   </si>
   <si>
     <t xml:space="preserve">CGP Pipeline Cross Application – mean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">same</t>
   </si>
   <si>
     <t xml:space="preserve">Running MAIPreform2_Spule0_0816_Upside_mean_pipeline on None) ...</t>
@@ -427,7 +424,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -472,31 +469,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -966,10 +943,10 @@
       <c r="M3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="0" t="n">
@@ -988,10 +965,10 @@
       <c r="M4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="0" t="n">
@@ -1010,10 +987,10 @@
       <c r="M5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="7" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="0" t="n">
@@ -1032,10 +1009,10 @@
       <c r="M6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="7" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="0" t="n">
@@ -1054,10 +1031,10 @@
       <c r="M7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="7" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="0" t="n">
@@ -1076,10 +1053,10 @@
       <c r="M8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="0" t="n">
@@ -1186,18 +1163,18 @@
       <c r="M13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="7" t="s">
         <v>31</v>
       </c>
       <c r="C14" s="0" t="n">
-        <v>0.2119</v>
+        <v>0.212</v>
       </c>
       <c r="D14" s="8" t="n">
         <f aca="false">B14-C14</f>
-        <v>0.035563260481127</v>
+        <v>0.035463260481127</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>10</v>
@@ -1670,18 +1647,18 @@
       <c r="M35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="13" t="n">
-        <v>0.60941</v>
+      <c r="C36" s="0" t="n">
+        <v>0.6094</v>
       </c>
       <c r="D36" s="8" t="n">
         <f aca="false">B36-C36</f>
-        <v>0.072540122424796</v>
+        <v>0.072550122424796</v>
       </c>
       <c r="G36" s="9" t="s">
         <v>10</v>
@@ -1758,10 +1735,10 @@
       <c r="M39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
+      <c r="A40" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="7" t="s">
         <v>83</v>
       </c>
       <c r="C40" s="0" t="n">
@@ -1873,13 +1850,13 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="12" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="6" t="s">
@@ -1904,7 +1881,7 @@
       <c r="B4" s="1" t="n">
         <v>0.0336391812216862</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="0" t="n">
         <v>0.0336</v>
       </c>
       <c r="D4" s="8" t="n">
@@ -1920,23 +1897,21 @@
       <c r="L4" s="10"/>
       <c r="M4" s="10"/>
       <c r="N4" s="10"/>
-      <c r="U4" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="6" t="n">
         <v>0.0332934765777646</v>
       </c>
-      <c r="C5" s="16" t="n">
-        <v>0.0091</v>
+      <c r="C5" s="0" t="n">
+        <v>0.0333</v>
       </c>
       <c r="D5" s="8" t="n">
         <f aca="false">B5-C5</f>
-        <v>0.0241934765777646</v>
+        <v>-6.52342223540076E-006</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>10</v>
@@ -1947,18 +1922,16 @@
       <c r="L5" s="10"/>
       <c r="M5" s="10"/>
       <c r="N5" s="10"/>
-      <c r="U5" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="6" t="n">
         <v>0.0336233839652003</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="0" t="n">
         <v>0.0336</v>
       </c>
       <c r="D6" s="8" t="n">
@@ -1974,18 +1947,16 @@
       <c r="L6" s="10"/>
       <c r="M6" s="10"/>
       <c r="N6" s="10"/>
-      <c r="U6" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="6" t="n">
         <v>0.124895082293055</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="0" t="n">
         <v>0.0686</v>
       </c>
       <c r="D7" s="8" t="n">
@@ -2001,18 +1972,16 @@
       <c r="L7" s="10"/>
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
-      <c r="U7" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="6" t="n">
         <v>0.126645067224404</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="0" t="n">
         <v>0.1271</v>
       </c>
       <c r="D8" s="8" t="n">
@@ -2028,18 +1997,16 @@
       <c r="L8" s="10"/>
       <c r="M8" s="10"/>
       <c r="N8" s="10"/>
-      <c r="U8" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="6" t="n">
         <v>0.23431241513234</v>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="0" t="n">
         <v>0.2382</v>
       </c>
       <c r="D9" s="8" t="n">
@@ -2055,18 +2022,16 @@
       <c r="L9" s="10"/>
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
-      <c r="U9" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="6" t="n">
         <v>0.0716789332816773</v>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="0" t="n">
         <v>0.0717</v>
       </c>
       <c r="D10" s="8" t="n">
@@ -2082,18 +2047,16 @@
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
       <c r="N10" s="10"/>
-      <c r="U10" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="6" t="n">
         <v>0.0752465163403073</v>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="0" t="n">
         <v>0.0752</v>
       </c>
       <c r="D11" s="8" t="n">
@@ -2109,18 +2072,16 @@
       <c r="L11" s="10"/>
       <c r="M11" s="10"/>
       <c r="N11" s="10"/>
-      <c r="U11" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="6" t="n">
         <v>0.131863378940609</v>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="0" t="n">
         <v>0.134</v>
       </c>
       <c r="D12" s="8" t="n">
@@ -2136,18 +2097,16 @@
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
-      <c r="U12" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="6" t="n">
         <v>0.129734882774295</v>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="0" t="n">
         <v>0.1309</v>
       </c>
       <c r="D13" s="8" t="n">
@@ -2163,18 +2122,16 @@
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
       <c r="N13" s="10"/>
-      <c r="U13" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="11" t="n">
+      <c r="B14" s="6" t="n">
         <v>0.634526773199268</v>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="0" t="n">
         <v>0.6331</v>
       </c>
       <c r="D14" s="8" t="n">
@@ -2190,18 +2147,16 @@
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
-      <c r="U14" s="1" t="s">
+      <c r="U14" s="1"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="B15" s="11" t="n">
+      <c r="B15" s="6" t="n">
         <v>0.218764576771259</v>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="C15" s="0" t="n">
         <v>0.2081</v>
       </c>
       <c r="D15" s="8" t="n">
@@ -2217,18 +2172,16 @@
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
-      <c r="U15" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="B16" s="11" t="n">
+      <c r="A16" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="6" t="n">
         <v>0.0794319310057269</v>
       </c>
-      <c r="C16" s="16" t="n">
+      <c r="C16" s="0" t="n">
         <v>0.0861</v>
       </c>
       <c r="D16" s="8" t="n">
@@ -2244,18 +2197,16 @@
       <c r="L16" s="10"/>
       <c r="M16" s="10"/>
       <c r="N16" s="10"/>
-      <c r="U16" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="6" t="n">
         <v>0.139515827407232</v>
       </c>
-      <c r="C17" s="16" t="n">
+      <c r="C17" s="0" t="n">
         <v>0.1438</v>
       </c>
       <c r="D17" s="8" t="n">
@@ -2271,18 +2222,16 @@
       <c r="L17" s="10"/>
       <c r="M17" s="10"/>
       <c r="N17" s="10"/>
-      <c r="U17" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="6" t="n">
         <v>0.150205554755411</v>
       </c>
-      <c r="C18" s="16" t="n">
+      <c r="C18" s="0" t="n">
         <v>0.1731</v>
       </c>
       <c r="D18" s="8" t="n">
@@ -2298,18 +2247,16 @@
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
       <c r="N18" s="10"/>
-      <c r="U18" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="6" t="n">
         <v>0.154036782755886</v>
       </c>
-      <c r="C19" s="16" t="n">
+      <c r="C19" s="0" t="n">
         <v>0.1205</v>
       </c>
       <c r="D19" s="8" t="n">
@@ -2325,18 +2272,16 @@
       <c r="L19" s="10"/>
       <c r="M19" s="10"/>
       <c r="N19" s="10"/>
-      <c r="U19" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="6" t="n">
         <v>0.355158537693472</v>
       </c>
-      <c r="C20" s="16" t="n">
+      <c r="C20" s="0" t="n">
         <v>0.3552</v>
       </c>
       <c r="D20" s="8" t="n">
@@ -2352,18 +2297,16 @@
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
       <c r="N20" s="10"/>
-      <c r="U20" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="6" t="n">
         <v>0.333674246249854</v>
       </c>
-      <c r="C21" s="16" t="n">
+      <c r="C21" s="0" t="n">
         <v>0.2454</v>
       </c>
       <c r="D21" s="8" t="n">
@@ -2380,25 +2323,22 @@
       <c r="L21" s="10"/>
       <c r="M21" s="10"/>
       <c r="N21" s="10"/>
-      <c r="U21" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U21" s="1"/>
     </row>
     <row r="22" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="6" t="n">
         <v>0.295085553531967</v>
       </c>
-      <c r="C22" s="16" t="n">
+      <c r="C22" s="0" t="n">
         <v>0.2951</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="8" t="n">
         <f aca="false">B22-C22</f>
         <v>-1.4446468032947E-005</v>
       </c>
-      <c r="E22" s="16"/>
       <c r="G22" s="9" t="s">
         <v>10</v>
       </c>
@@ -2408,18 +2348,16 @@
       <c r="L22" s="10"/>
       <c r="M22" s="10"/>
       <c r="N22" s="10"/>
-      <c r="U22" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B23" s="1" t="n">
         <v>0.85641154944387</v>
       </c>
-      <c r="C23" s="16" t="n">
+      <c r="C23" s="0" t="n">
         <v>0.8707</v>
       </c>
       <c r="D23" s="8" t="n">
@@ -2435,18 +2373,16 @@
       <c r="L23" s="10"/>
       <c r="M23" s="10"/>
       <c r="N23" s="10"/>
-      <c r="U23" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U23" s="1"/>
     </row>
     <row r="24" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="11" t="n">
+      <c r="B24" s="6" t="n">
         <v>0.121245169346358</v>
       </c>
-      <c r="C24" s="16" t="n">
+      <c r="C24" s="0" t="n">
         <v>0.1212</v>
       </c>
       <c r="D24" s="8" t="n">
@@ -2462,18 +2398,16 @@
       <c r="L24" s="10"/>
       <c r="M24" s="10"/>
       <c r="N24" s="10"/>
-      <c r="U24" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U24" s="1"/>
     </row>
     <row r="25" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="11" t="n">
+      <c r="B25" s="6" t="n">
         <v>0.0982267970643694</v>
       </c>
-      <c r="C25" s="16" t="n">
+      <c r="C25" s="0" t="n">
         <v>0.0523</v>
       </c>
       <c r="D25" s="8" t="n">
@@ -2489,18 +2423,16 @@
       <c r="L25" s="10"/>
       <c r="M25" s="10"/>
       <c r="N25" s="10"/>
-      <c r="U25" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U25" s="1"/>
     </row>
     <row r="26" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="11" t="n">
+      <c r="B26" s="6" t="n">
         <v>0.447453831653456</v>
       </c>
-      <c r="C26" s="16" t="n">
+      <c r="C26" s="0" t="n">
         <v>0.4475</v>
       </c>
       <c r="D26" s="8" t="n">
@@ -2516,18 +2448,16 @@
       <c r="L26" s="10"/>
       <c r="M26" s="10"/>
       <c r="N26" s="10"/>
-      <c r="U26" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="11" t="n">
+      <c r="B27" s="6" t="n">
         <v>0.460727494072827</v>
       </c>
-      <c r="C27" s="16" t="n">
+      <c r="C27" s="0" t="n">
         <v>0.4607</v>
       </c>
       <c r="D27" s="8" t="n">
@@ -2543,23 +2473,21 @@
       <c r="L27" s="10"/>
       <c r="M27" s="10"/>
       <c r="N27" s="10"/>
-      <c r="U27" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="B28" s="11" t="n">
+      <c r="A28" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="6" t="n">
         <v>0.385139499824248</v>
       </c>
-      <c r="C28" s="16" t="n">
-        <v>0.3219</v>
+      <c r="C28" s="0" t="n">
+        <v>0.3681</v>
       </c>
       <c r="D28" s="8" t="n">
         <f aca="false">B28-C28</f>
-        <v>0.063239499824248</v>
+        <v>0.017039499824248</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>10</v>
@@ -2570,23 +2498,21 @@
       <c r="L28" s="10"/>
       <c r="M28" s="10"/>
       <c r="N28" s="10"/>
-      <c r="U28" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="16" t="n">
+      <c r="B29" s="1" t="n">
         <v>0.121244975869924</v>
       </c>
-      <c r="C29" s="16" t="n">
-        <v>0.0558</v>
+      <c r="C29" s="0" t="n">
+        <v>0.1207</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">B29-C29</f>
-        <v>0.065444975869924</v>
+        <v>0.000544975869923997</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>10</v>
@@ -2597,18 +2523,16 @@
       <c r="L29" s="10"/>
       <c r="M29" s="10"/>
       <c r="N29" s="10"/>
-      <c r="U29" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U29" s="1"/>
     </row>
     <row r="30" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="11" t="n">
+      <c r="B30" s="6" t="n">
         <v>0.545694298252736</v>
       </c>
-      <c r="C30" s="16" t="n">
+      <c r="C30" s="0" t="n">
         <v>0.5457</v>
       </c>
       <c r="D30" s="8" t="n">
@@ -2624,18 +2548,16 @@
       <c r="L30" s="10"/>
       <c r="M30" s="10"/>
       <c r="N30" s="10"/>
-      <c r="U30" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U30" s="1"/>
     </row>
     <row r="31" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="11" t="n">
+      <c r="B31" s="6" t="n">
         <v>0.193653302161922</v>
       </c>
-      <c r="C31" s="16" t="n">
+      <c r="C31" s="0" t="n">
         <v>0.1937</v>
       </c>
       <c r="D31" s="8" t="n">
@@ -2651,18 +2573,16 @@
       <c r="L31" s="10"/>
       <c r="M31" s="10"/>
       <c r="N31" s="10"/>
-      <c r="U31" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U31" s="1"/>
     </row>
     <row r="32" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B32" s="16" t="n">
+      <c r="B32" s="1" t="n">
         <v>0.571710499739276</v>
       </c>
-      <c r="C32" s="16" t="n">
+      <c r="C32" s="0" t="n">
         <v>0.5657</v>
       </c>
       <c r="D32" s="8" t="n">
@@ -2678,18 +2598,16 @@
       <c r="L32" s="10"/>
       <c r="M32" s="10"/>
       <c r="N32" s="10"/>
-      <c r="U32" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U32" s="1"/>
     </row>
     <row r="33" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16" t="s">
+      <c r="A33" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B33" s="16" t="n">
+      <c r="B33" s="1" t="n">
         <v>0.206353390389513</v>
       </c>
-      <c r="C33" s="16" t="n">
+      <c r="C33" s="0" t="n">
         <v>0.2061</v>
       </c>
       <c r="D33" s="8" t="n">
@@ -2705,18 +2623,16 @@
       <c r="L33" s="10"/>
       <c r="M33" s="10"/>
       <c r="N33" s="10"/>
-      <c r="U33" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U33" s="1"/>
     </row>
     <row r="34" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B34" s="16" t="n">
+      <c r="B34" s="1" t="n">
         <v>0.553598109256054</v>
       </c>
-      <c r="C34" s="16" t="n">
+      <c r="C34" s="0" t="n">
         <v>0.5536</v>
       </c>
       <c r="D34" s="8" t="n">
@@ -2732,18 +2648,16 @@
       <c r="L34" s="10"/>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
-      <c r="U34" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U34" s="1"/>
     </row>
     <row r="35" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B35" s="6" t="n">
         <v>0.321007485833355</v>
       </c>
-      <c r="C35" s="16" t="n">
+      <c r="C35" s="0" t="n">
         <v>0.321</v>
       </c>
       <c r="D35" s="8" t="n">
@@ -2759,18 +2673,16 @@
       <c r="L35" s="10"/>
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
-      <c r="U35" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U35" s="1"/>
     </row>
     <row r="36" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B36" s="11" t="n">
+      <c r="B36" s="6" t="n">
         <v>0.396820538135367</v>
       </c>
-      <c r="C36" s="16" t="n">
+      <c r="C36" s="0" t="n">
         <v>0.3968</v>
       </c>
       <c r="D36" s="8" t="n">
@@ -2786,18 +2698,16 @@
       <c r="L36" s="10"/>
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
-      <c r="U36" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U36" s="1"/>
     </row>
     <row r="37" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
+      <c r="A37" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="11" t="n">
+      <c r="B37" s="6" t="n">
         <v>0.633261326857541</v>
       </c>
-      <c r="C37" s="16" t="n">
+      <c r="C37" s="0" t="n">
         <v>0.6387</v>
       </c>
       <c r="D37" s="8" t="n">
@@ -2813,18 +2723,16 @@
       <c r="L37" s="10"/>
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
-      <c r="U37" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U37" s="1"/>
     </row>
     <row r="38" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B38" s="11" t="n">
+      <c r="A38" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B38" s="6" t="n">
         <v>0.728388899750556</v>
       </c>
-      <c r="C38" s="16" t="n">
+      <c r="C38" s="0" t="n">
         <v>0.7284</v>
       </c>
       <c r="D38" s="8" t="n">
@@ -2840,18 +2748,16 @@
       <c r="L38" s="10"/>
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>
-      <c r="U38" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U38" s="1"/>
     </row>
     <row r="39" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="B39" s="11" t="n">
+      <c r="A39" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B39" s="6" t="n">
         <v>0.210338073888041</v>
       </c>
-      <c r="C39" s="16" t="n">
+      <c r="C39" s="0" t="n">
         <v>0.2002</v>
       </c>
       <c r="D39" s="8" t="n">
@@ -2867,16 +2773,14 @@
       <c r="L39" s="10"/>
       <c r="M39" s="10"/>
       <c r="N39" s="10"/>
-      <c r="U39" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U39" s="1"/>
     </row>
     <row r="40" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B40" s="6"/>
-      <c r="C40" s="1" t="n">
+      <c r="C40" s="0" t="n">
         <v>0.3386</v>
       </c>
       <c r="D40" s="8" t="n">
@@ -2892,16 +2796,14 @@
       <c r="L40" s="10"/>
       <c r="M40" s="10"/>
       <c r="N40" s="10"/>
-      <c r="U40" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U40" s="1"/>
     </row>
     <row r="41" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B41" s="6"/>
-      <c r="C41" s="1" t="n">
+      <c r="C41" s="0" t="n">
         <v>0.2093</v>
       </c>
       <c r="D41" s="8" t="n">
@@ -2917,9 +2819,7 @@
       <c r="L41" s="10"/>
       <c r="M41" s="10"/>
       <c r="N41" s="10"/>
-      <c r="U41" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="U41" s="1"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G42" s="6"/>

</xml_diff>

<commit_message>
Fix WStep because Width variable was not right
</commit_message>
<xml_diff>
--- a/param_tuning/20250927-datasets.xlsx
+++ b/param_tuning/20250927-datasets.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Best" sheetId="1" state="visible" r:id="rId3"/>
@@ -1170,11 +1170,11 @@
         <v>31</v>
       </c>
       <c r="C14" s="0" t="n">
-        <v>0.212</v>
+        <v>0.2093</v>
       </c>
       <c r="D14" s="8" t="n">
         <f aca="false">B14-C14</f>
-        <v>0.035463260481127</v>
+        <v>0.038163260481127</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>10</v>
@@ -1412,11 +1412,11 @@
         <v>53</v>
       </c>
       <c r="C25" s="0" t="n">
-        <v>0.4741</v>
+        <v>0.3749</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">B25-C25</f>
-        <v>-3.98283286501266E-006</v>
+        <v>0.099196017167135</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>10</v>
@@ -1478,11 +1478,11 @@
         <v>59</v>
       </c>
       <c r="C28" s="0" t="n">
-        <v>0.0688</v>
+        <v>0.098</v>
       </c>
       <c r="D28" s="8" t="n">
         <f aca="false">B28-C28</f>
-        <v>0.069270422673154</v>
+        <v>0.040070422673154</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>10</v>
@@ -1500,11 +1500,11 @@
         <v>61</v>
       </c>
       <c r="C29" s="0" t="n">
-        <v>0.589</v>
+        <v>0.571</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">B29-C29</f>
-        <v>0.00137942095130905</v>
+        <v>0.0193794209513091</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>10</v>
@@ -1676,11 +1676,11 @@
         <v>77</v>
       </c>
       <c r="C37" s="0" t="n">
-        <v>0.7284</v>
+        <v>0.714</v>
       </c>
       <c r="D37" s="8" t="n">
         <f aca="false">B37-C37</f>
-        <v>-0.0219720789680481</v>
+        <v>-0.00757207896804801</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>10</v>
@@ -2508,11 +2508,11 @@
         <v>0.121244975869924</v>
       </c>
       <c r="C29" s="0" t="n">
-        <v>0.1207</v>
+        <v>0.1185</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">B29-C29</f>
-        <v>0.000544975869923997</v>
+        <v>0.002744975869924</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>10</v>

</xml_diff>